<commit_message>
Sync local state: updated scripts, new templates, PS1 utilities, price lists, output files
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/sales_item_match_audit.xlsx
+++ b/outputs/sales_item_match_audit.xlsx
@@ -23806,12 +23806,12 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.419</t>
         </is>
       </c>
       <c r="P180" t="inlineStr"/>
@@ -23821,17 +23821,17 @@
       <c r="T180" t="inlineStr"/>
       <c r="U180" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="V180" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>T-Shaped Rubber, 18"</t>
         </is>
       </c>
       <c r="X180" t="inlineStr">
@@ -23846,19 +23846,59 @@
       </c>
       <c r="Z180" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AA180" t="inlineStr"/>
-      <c r="AB180" t="inlineStr"/>
-      <c r="AC180" t="inlineStr"/>
-      <c r="AD180" t="inlineStr"/>
-      <c r="AE180" t="inlineStr"/>
-      <c r="AF180" t="inlineStr"/>
-      <c r="AG180" t="inlineStr"/>
-      <c r="AH180" t="inlineStr"/>
-      <c r="AI180" t="inlineStr"/>
-      <c r="AJ180" t="inlineStr"/>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AA180" t="inlineStr">
+        <is>
+          <t>0.419</t>
+        </is>
+      </c>
+      <c r="AB180" t="inlineStr">
+        <is>
+          <t>Ettore Sleeve Pro+ Microfiber 18 inch</t>
+        </is>
+      </c>
+      <c r="AC180" t="inlineStr">
+        <is>
+          <t>40018</t>
+        </is>
+      </c>
+      <c r="AD180" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE180" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF180" t="inlineStr">
+        <is>
+          <t>0.415</t>
+        </is>
+      </c>
+      <c r="AG180" t="inlineStr">
+        <is>
+          <t>Ettore Squeegee Complete 18</t>
+        </is>
+      </c>
+      <c r="AH180" t="inlineStr">
+        <is>
+          <t>JRACEN-MASTER-BRASS-SQUEEGEES-COMPLET-3</t>
+        </is>
+      </c>
+      <c r="AI180" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ180" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -25779,7 +25819,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>0.437</t>
+          <t>0.426</t>
         </is>
       </c>
       <c r="P194" t="inlineStr"/>
@@ -25819,17 +25859,17 @@
       </c>
       <c r="AA194" t="inlineStr">
         <is>
-          <t>0.437</t>
+          <t>0.426</t>
         </is>
       </c>
       <c r="AB194" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Ettore T-Bar ProGrip 18 inch</t>
         </is>
       </c>
       <c r="AC194" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-PRO-GRIP-T-BAR-18</t>
         </is>
       </c>
       <c r="AD194" t="inlineStr">
@@ -25839,32 +25879,32 @@
       </c>
       <c r="AE194" t="inlineStr">
         <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF194" t="inlineStr">
+        <is>
+          <t>0.419</t>
+        </is>
+      </c>
+      <c r="AG194" t="inlineStr">
+        <is>
+          <t>Ettore Channel Classic Aluminum 18 inch</t>
+        </is>
+      </c>
+      <c r="AH194" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="AI194" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ194" t="inlineStr">
+        <is>
           <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AF194" t="inlineStr">
-        <is>
-          <t>0.426</t>
-        </is>
-      </c>
-      <c r="AG194" t="inlineStr">
-        <is>
-          <t>Ettore T-Bar ProGrip 18 inch</t>
-        </is>
-      </c>
-      <c r="AH194" t="inlineStr">
-        <is>
-          <t>JRACEN-PRO-GRIP-T-BAR-18</t>
-        </is>
-      </c>
-      <c r="AI194" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AJ194" t="inlineStr">
-        <is>
-          <t>1 shared tokens, category fit</t>
         </is>
       </c>
     </row>
@@ -28972,12 +29012,12 @@
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.371</t>
         </is>
       </c>
       <c r="P217" t="inlineStr"/>
@@ -28987,17 +29027,17 @@
       <c r="T217" t="inlineStr"/>
       <c r="U217" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="V217" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="W217" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 30 inch</t>
+          <t>T-Shaped Rubber, 30"</t>
         </is>
       </c>
       <c r="X217" t="inlineStr">
@@ -29012,19 +29052,59 @@
       </c>
       <c r="Z217" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AA217" t="inlineStr"/>
-      <c r="AB217" t="inlineStr"/>
-      <c r="AC217" t="inlineStr"/>
-      <c r="AD217" t="inlineStr"/>
-      <c r="AE217" t="inlineStr"/>
-      <c r="AF217" t="inlineStr"/>
-      <c r="AG217" t="inlineStr"/>
-      <c r="AH217" t="inlineStr"/>
-      <c r="AI217" t="inlineStr"/>
-      <c r="AJ217" t="inlineStr"/>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AA217" t="inlineStr">
+        <is>
+          <t>0.371</t>
+        </is>
+      </c>
+      <c r="AB217" t="inlineStr">
+        <is>
+          <t>Aluminum Floor Squeegees, Straight, 30"</t>
+        </is>
+      </c>
+      <c r="AC217" t="inlineStr">
+        <is>
+          <t>55030</t>
+        </is>
+      </c>
+      <c r="AD217" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE217" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF217" t="inlineStr">
+        <is>
+          <t>0.361</t>
+        </is>
+      </c>
+      <c r="AG217" t="inlineStr">
+        <is>
+          <t>Ettore Super Channel Aluminum 30 inch</t>
+        </is>
+      </c>
+      <c r="AH217" t="inlineStr">
+        <is>
+          <t>11040</t>
+        </is>
+      </c>
+      <c r="AI217" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ217" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -31999,7 +32079,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>0.355</t>
+          <t>0.312</t>
         </is>
       </c>
       <c r="P238" t="inlineStr"/>
@@ -32039,17 +32119,17 @@
       </c>
       <c r="AA238" t="inlineStr">
         <is>
-          <t>0.355</t>
+          <t>0.312</t>
         </is>
       </c>
       <c r="AB238" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>T-Shaped Rubber, 36"</t>
         </is>
       </c>
       <c r="AC238" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>1521</t>
         </is>
       </c>
       <c r="AD238" t="inlineStr">
@@ -32059,22 +32139,22 @@
       </c>
       <c r="AE238" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="AF238" t="inlineStr">
         <is>
-          <t>0.355</t>
+          <t>0.312</t>
         </is>
       </c>
       <c r="AG238" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 36 inch</t>
+          <t>T-Shaped Rubber, 30"</t>
         </is>
       </c>
       <c r="AH238" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>1518</t>
         </is>
       </c>
       <c r="AI238" t="inlineStr">
@@ -32084,7 +32164,7 @@
       </c>
       <c r="AJ238" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
     </row>
@@ -34275,7 +34355,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>0.261</t>
+          <t>0.231</t>
         </is>
       </c>
       <c r="P254" t="inlineStr"/>
@@ -34315,17 +34395,17 @@
       </c>
       <c r="AA254" t="inlineStr">
         <is>
-          <t>0.261</t>
+          <t>0.231</t>
         </is>
       </c>
       <c r="AB254" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 14 inch [Case 36]</t>
         </is>
       </c>
       <c r="AC254" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-8</t>
         </is>
       </c>
       <c r="AD254" t="inlineStr">
@@ -34340,17 +34420,17 @@
       </c>
       <c r="AF254" t="inlineStr">
         <is>
-          <t>0.248</t>
+          <t>0.231</t>
         </is>
       </c>
       <c r="AG254" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 36 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 06 inch [Case 36]</t>
         </is>
       </c>
       <c r="AH254" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-6</t>
         </is>
       </c>
       <c r="AI254" t="inlineStr">
@@ -34432,12 +34512,12 @@
       </c>
       <c r="N255" t="inlineStr">
         <is>
-          <t>0.420</t>
+          <t>0.310</t>
         </is>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>0.420</t>
+          <t>0.306</t>
         </is>
       </c>
       <c r="P255" t="inlineStr"/>
@@ -34447,22 +34527,22 @@
       <c r="T255" t="inlineStr"/>
       <c r="U255" t="inlineStr">
         <is>
-          <t>3 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="V255" t="inlineStr">
         <is>
-          <t>0.420</t>
+          <t>0.310</t>
         </is>
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 36 inch</t>
+          <t>Ettore Pole Replacement Grip 3rd</t>
         </is>
       </c>
       <c r="X255" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>JRACEN-REPLACEMENT-GRIPS-3-SEC</t>
         </is>
       </c>
       <c r="Y255" t="inlineStr">
@@ -34472,22 +34552,22 @@
       </c>
       <c r="Z255" t="inlineStr">
         <is>
-          <t>3 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="AA255" t="inlineStr">
         <is>
-          <t>0.420</t>
+          <t>0.306</t>
         </is>
       </c>
       <c r="AB255" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 30 inch</t>
+          <t>Ettore Rubber Master Replacement Dozen 08 inch</t>
         </is>
       </c>
       <c r="AC255" t="inlineStr">
         <is>
-          <t>1518</t>
+          <t>JRACEN-MASTER-RUBBER-8</t>
         </is>
       </c>
       <c r="AD255" t="inlineStr">
@@ -34497,22 +34577,22 @@
       </c>
       <c r="AE255" t="inlineStr">
         <is>
-          <t>3 shared tokens, category fit</t>
+          <t>2 shared tokens, category fit</t>
         </is>
       </c>
       <c r="AF255" t="inlineStr">
         <is>
-          <t>0.420</t>
+          <t>0.306</t>
         </is>
       </c>
       <c r="AG255" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 24 inch</t>
+          <t>Ettore Rubber Master Replacement Dozen 06 inch</t>
         </is>
       </c>
       <c r="AH255" t="inlineStr">
         <is>
-          <t>1512</t>
+          <t>JRACEN-MASTER-RUBBER-6</t>
         </is>
       </c>
       <c r="AI255" t="inlineStr">
@@ -34522,7 +34602,7 @@
       </c>
       <c r="AJ255" t="inlineStr">
         <is>
-          <t>3 shared tokens, category fit</t>
+          <t>2 shared tokens, category fit</t>
         </is>
       </c>
     </row>
@@ -35588,12 +35668,12 @@
       </c>
       <c r="N263" t="inlineStr">
         <is>
-          <t>0.358</t>
+          <t>0.344</t>
         </is>
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>0.344</t>
+          <t>0.337</t>
         </is>
       </c>
       <c r="P263" t="inlineStr"/>
@@ -35608,67 +35688,67 @@
       </c>
       <c r="V263" t="inlineStr">
         <is>
-          <t>0.358</t>
+          <t>0.344</t>
         </is>
       </c>
       <c r="W263" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 22 inch</t>
+          <t>Ettore Rubber Master Replacement Gross 22 inch [Case 144]</t>
         </is>
       </c>
       <c r="X263" t="inlineStr">
         <is>
+          <t>JRACEN-MASTER-RUBBER-22-CASE-144</t>
+        </is>
+      </c>
+      <c r="Y263" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="Z263" t="inlineStr">
+        <is>
+          <t>2 shared tokens</t>
+        </is>
+      </c>
+      <c r="AA263" t="inlineStr">
+        <is>
+          <t>0.337</t>
+        </is>
+      </c>
+      <c r="AB263" t="inlineStr">
+        <is>
+          <t>Ettore Rubber Master Replacement Dozen 22 inch [Case 12]</t>
+        </is>
+      </c>
+      <c r="AC263" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="AD263" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE263" t="inlineStr">
+        <is>
+          <t>2 shared tokens</t>
+        </is>
+      </c>
+      <c r="AF263" t="inlineStr">
+        <is>
+          <t>0.321</t>
+        </is>
+      </c>
+      <c r="AG263" t="inlineStr">
+        <is>
+          <t>T-Shaped Rubber, 22"</t>
+        </is>
+      </c>
+      <c r="AH263" t="inlineStr">
+        <is>
           <t>JRACEN-T-SHAPED-RUBBER-22</t>
-        </is>
-      </c>
-      <c r="Y263" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="Z263" t="inlineStr">
-        <is>
-          <t>2 shared tokens</t>
-        </is>
-      </c>
-      <c r="AA263" t="inlineStr">
-        <is>
-          <t>0.344</t>
-        </is>
-      </c>
-      <c r="AB263" t="inlineStr">
-        <is>
-          <t>Ettore Rubber Master Replacement Gross 22 inch [Case 144]</t>
-        </is>
-      </c>
-      <c r="AC263" t="inlineStr">
-        <is>
-          <t>JRACEN-MASTER-RUBBER-22-CASE-144</t>
-        </is>
-      </c>
-      <c r="AD263" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AE263" t="inlineStr">
-        <is>
-          <t>2 shared tokens</t>
-        </is>
-      </c>
-      <c r="AF263" t="inlineStr">
-        <is>
-          <t>0.337</t>
-        </is>
-      </c>
-      <c r="AG263" t="inlineStr">
-        <is>
-          <t>Ettore Rubber Master Replacement Dozen 22 inch [Case 12]</t>
-        </is>
-      </c>
-      <c r="AH263" t="inlineStr">
-        <is>
-          <t>1438</t>
         </is>
       </c>
       <c r="AI263" t="inlineStr">
@@ -36940,12 +37020,12 @@
       </c>
       <c r="N273" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.329</t>
         </is>
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>0.329</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="P273" t="inlineStr"/>
@@ -36960,17 +37040,17 @@
       </c>
       <c r="V273" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.329</t>
         </is>
       </c>
       <c r="W273" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 14 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 14 inch [Case 36]</t>
         </is>
       </c>
       <c r="X273" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-8</t>
         </is>
       </c>
       <c r="Y273" t="inlineStr">
@@ -36983,31 +37063,11 @@
           <t>2 shared tokens, category fit</t>
         </is>
       </c>
-      <c r="AA273" t="inlineStr">
-        <is>
-          <t>0.329</t>
-        </is>
-      </c>
-      <c r="AB273" t="inlineStr">
-        <is>
-          <t>Sorbo Channel Ultralight w/End Clip 14 inch [Case 36]</t>
-        </is>
-      </c>
-      <c r="AC273" t="inlineStr">
-        <is>
-          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-8</t>
-        </is>
-      </c>
-      <c r="AD273" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AE273" t="inlineStr">
-        <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
+      <c r="AA273" t="inlineStr"/>
+      <c r="AB273" t="inlineStr"/>
+      <c r="AC273" t="inlineStr"/>
+      <c r="AD273" t="inlineStr"/>
+      <c r="AE273" t="inlineStr"/>
       <c r="AF273" t="inlineStr"/>
       <c r="AG273" t="inlineStr"/>
       <c r="AH273" t="inlineStr"/>
@@ -41995,7 +42055,7 @@
       </c>
       <c r="O308" t="inlineStr">
         <is>
-          <t>0.355</t>
+          <t>0.312</t>
         </is>
       </c>
       <c r="P308" t="inlineStr"/>
@@ -42035,17 +42095,17 @@
       </c>
       <c r="AA308" t="inlineStr">
         <is>
-          <t>0.355</t>
+          <t>0.312</t>
         </is>
       </c>
       <c r="AB308" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>T-Shaped Rubber, 36"</t>
         </is>
       </c>
       <c r="AC308" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>1521</t>
         </is>
       </c>
       <c r="AD308" t="inlineStr">
@@ -42055,22 +42115,22 @@
       </c>
       <c r="AE308" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="AF308" t="inlineStr">
         <is>
-          <t>0.355</t>
+          <t>0.312</t>
         </is>
       </c>
       <c r="AG308" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 36 inch</t>
+          <t>T-Shaped Rubber, 30"</t>
         </is>
       </c>
       <c r="AH308" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>1518</t>
         </is>
       </c>
       <c r="AI308" t="inlineStr">
@@ -42080,7 +42140,7 @@
       </c>
       <c r="AJ308" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
     </row>
@@ -44171,7 +44231,7 @@
       </c>
       <c r="O324" t="inlineStr">
         <is>
-          <t>0.437</t>
+          <t>0.386</t>
         </is>
       </c>
       <c r="P324" t="inlineStr"/>
@@ -44211,42 +44271,42 @@
       </c>
       <c r="AA324" t="inlineStr">
         <is>
-          <t>0.437</t>
+          <t>0.386</t>
         </is>
       </c>
       <c r="AB324" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 24 inch</t>
+          <t>Super Channel 14"</t>
         </is>
       </c>
       <c r="AC324" t="inlineStr">
         <is>
+          <t>JRACEN-SUPER-CHANNEL-14</t>
+        </is>
+      </c>
+      <c r="AD324" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE324" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF324" t="inlineStr">
+        <is>
+          <t>0.373</t>
+        </is>
+      </c>
+      <c r="AG324" t="inlineStr">
+        <is>
+          <t>T-Shaped Rubber, 24"</t>
+        </is>
+      </c>
+      <c r="AH324" t="inlineStr">
+        <is>
           <t>1512</t>
-        </is>
-      </c>
-      <c r="AD324" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AE324" t="inlineStr">
-        <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AF324" t="inlineStr">
-        <is>
-          <t>0.386</t>
-        </is>
-      </c>
-      <c r="AG324" t="inlineStr">
-        <is>
-          <t>Super Channel 14"</t>
-        </is>
-      </c>
-      <c r="AH324" t="inlineStr">
-        <is>
-          <t>JRACEN-SUPER-CHANNEL-14</t>
         </is>
       </c>
       <c r="AI324" t="inlineStr">
@@ -47740,12 +47800,12 @@
       </c>
       <c r="N349" t="inlineStr">
         <is>
-          <t>0.550</t>
+          <t>0.484</t>
         </is>
       </c>
       <c r="O349" t="inlineStr">
         <is>
-          <t>0.484</t>
+          <t>0.408</t>
         </is>
       </c>
       <c r="P349" t="inlineStr"/>
@@ -47760,17 +47820,17 @@
       </c>
       <c r="V349" t="inlineStr">
         <is>
-          <t>0.550</t>
+          <t>0.484</t>
         </is>
       </c>
       <c r="W349" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Ettore Rubber Master Replacement Dozen 18 inch [Case 12]</t>
         </is>
       </c>
       <c r="X349" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-MASTER-RUBBER-18-CASE-12</t>
         </is>
       </c>
       <c r="Y349" t="inlineStr">
@@ -47785,17 +47845,17 @@
       </c>
       <c r="AA349" t="inlineStr">
         <is>
-          <t>0.484</t>
+          <t>0.408</t>
         </is>
       </c>
       <c r="AB349" t="inlineStr">
         <is>
-          <t>Ettore Rubber Master Replacement Dozen 18 inch [Case 12]</t>
+          <t>Ettore Rubber Master Replacement Dozen 12 inch [Case 12]</t>
         </is>
       </c>
       <c r="AC349" t="inlineStr">
         <is>
-          <t>JRACEN-MASTER-RUBBER-18-CASE-12</t>
+          <t>JRACEN-MASTER-RUBBER-12-CASE-12</t>
         </is>
       </c>
       <c r="AD349" t="inlineStr">
@@ -47805,22 +47865,22 @@
       </c>
       <c r="AE349" t="inlineStr">
         <is>
-          <t>4 shared tokens, category fit</t>
+          <t>3 shared tokens, category fit</t>
         </is>
       </c>
       <c r="AF349" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.397</t>
         </is>
       </c>
       <c r="AG349" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 24 inch</t>
+          <t>Ettore Rubber Master Replacement Gross 12 inch [Case 144]</t>
         </is>
       </c>
       <c r="AH349" t="inlineStr">
         <is>
-          <t>1512</t>
+          <t>JRACEN-MASTER-RUBBER-12-CASE-144</t>
         </is>
       </c>
       <c r="AI349" t="inlineStr">
@@ -50988,12 +51048,12 @@
       </c>
       <c r="N373" t="inlineStr">
         <is>
-          <t>0.312</t>
+          <t>0.300</t>
         </is>
       </c>
       <c r="O373" t="inlineStr">
         <is>
-          <t>0.301</t>
+          <t>0.288</t>
         </is>
       </c>
       <c r="P373" t="inlineStr"/>
@@ -51008,17 +51068,17 @@
       </c>
       <c r="V373" t="inlineStr">
         <is>
-          <t>0.312</t>
+          <t>0.300</t>
         </is>
       </c>
       <c r="W373" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Ettore Sleeve Dura 22 inch</t>
         </is>
       </c>
       <c r="X373" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="Y373" t="inlineStr">
@@ -51033,17 +51093,17 @@
       </c>
       <c r="AA373" t="inlineStr">
         <is>
-          <t>0.301</t>
+          <t>0.288</t>
         </is>
       </c>
       <c r="AB373" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 22 inch</t>
+          <t>Ettore Sleeve Dura 18 inch</t>
         </is>
       </c>
       <c r="AC373" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-22</t>
+          <t>JRACEN-DURA-2-SLEEVE-18</t>
         </is>
       </c>
       <c r="AD373" t="inlineStr">
@@ -51058,17 +51118,17 @@
       </c>
       <c r="AF373" t="inlineStr">
         <is>
-          <t>0.300</t>
+          <t>0.288</t>
         </is>
       </c>
       <c r="AG373" t="inlineStr">
         <is>
-          <t>Ettore Sleeve Dura 22 inch</t>
+          <t>Ettore Sleeve Dura 14 inch</t>
         </is>
       </c>
       <c r="AH373" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1880</t>
         </is>
       </c>
       <c r="AI373" t="inlineStr">
@@ -52434,7 +52494,7 @@
       </c>
       <c r="N384" t="inlineStr">
         <is>
-          <t>0.445</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="O384" t="inlineStr">
@@ -52454,12 +52514,12 @@
       </c>
       <c r="V384" t="inlineStr">
         <is>
-          <t>0.445</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="W384" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>T-Shaped Rubber, 18"</t>
         </is>
       </c>
       <c r="X384" t="inlineStr">
@@ -55948,12 +56008,12 @@
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t>0.398</t>
+          <t>0.384</t>
         </is>
       </c>
       <c r="O409" t="inlineStr">
         <is>
-          <t>0.384</t>
+          <t>0.377</t>
         </is>
       </c>
       <c r="P409" t="inlineStr"/>
@@ -55968,67 +56028,67 @@
       </c>
       <c r="V409" t="inlineStr">
         <is>
-          <t>0.398</t>
+          <t>0.384</t>
         </is>
       </c>
       <c r="W409" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 14 inch</t>
+          <t>Ettore Rubber Master Replacement Gross 14 inch [Case 144]</t>
         </is>
       </c>
       <c r="X409" t="inlineStr">
         <is>
+          <t>JRACEN-MASTER-RUBBER-14-CASE-144</t>
+        </is>
+      </c>
+      <c r="Y409" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="Z409" t="inlineStr">
+        <is>
+          <t>2 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AA409" t="inlineStr">
+        <is>
+          <t>0.377</t>
+        </is>
+      </c>
+      <c r="AB409" t="inlineStr">
+        <is>
+          <t>Ettore Rubber Master Replacement Dozen 14 inch [Case 12]</t>
+        </is>
+      </c>
+      <c r="AC409" t="inlineStr">
+        <is>
+          <t>JRACEN-MASTER-RUBBER-14-CASE-12</t>
+        </is>
+      </c>
+      <c r="AD409" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE409" t="inlineStr">
+        <is>
+          <t>2 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF409" t="inlineStr">
+        <is>
+          <t>0.361</t>
+        </is>
+      </c>
+      <c r="AG409" t="inlineStr">
+        <is>
+          <t>T-Shaped Rubber, 14"</t>
+        </is>
+      </c>
+      <c r="AH409" t="inlineStr">
+        <is>
           <t>1497</t>
-        </is>
-      </c>
-      <c r="Y409" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="Z409" t="inlineStr">
-        <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AA409" t="inlineStr">
-        <is>
-          <t>0.384</t>
-        </is>
-      </c>
-      <c r="AB409" t="inlineStr">
-        <is>
-          <t>Ettore Rubber Master Replacement Gross 14 inch [Case 144]</t>
-        </is>
-      </c>
-      <c r="AC409" t="inlineStr">
-        <is>
-          <t>JRACEN-MASTER-RUBBER-14-CASE-144</t>
-        </is>
-      </c>
-      <c r="AD409" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AE409" t="inlineStr">
-        <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AF409" t="inlineStr">
-        <is>
-          <t>0.377</t>
-        </is>
-      </c>
-      <c r="AG409" t="inlineStr">
-        <is>
-          <t>Ettore Rubber Master Replacement Dozen 14 inch [Case 12]</t>
-        </is>
-      </c>
-      <c r="AH409" t="inlineStr">
-        <is>
-          <t>JRACEN-MASTER-RUBBER-14-CASE-12</t>
         </is>
       </c>
       <c r="AI409" t="inlineStr">
@@ -57621,7 +57681,7 @@
       </c>
       <c r="O421" t="inlineStr">
         <is>
-          <t>0.312</t>
+          <t>0.300</t>
         </is>
       </c>
       <c r="P421" t="inlineStr"/>
@@ -57661,17 +57721,17 @@
       </c>
       <c r="AA421" t="inlineStr">
         <is>
-          <t>0.312</t>
+          <t>0.300</t>
         </is>
       </c>
       <c r="AB421" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Ettore Sleeve Dura 14 inch</t>
         </is>
       </c>
       <c r="AC421" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>1880</t>
         </is>
       </c>
       <c r="AD421" t="inlineStr">
@@ -57686,17 +57746,17 @@
       </c>
       <c r="AF421" t="inlineStr">
         <is>
-          <t>0.301</t>
+          <t>0.295</t>
         </is>
       </c>
       <c r="AG421" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 14 inch</t>
+          <t>Ettore Sleeve Mighty 14 inch</t>
         </is>
       </c>
       <c r="AH421" t="inlineStr">
         <is>
-          <t>1497</t>
+          <t>52014</t>
         </is>
       </c>
       <c r="AI421" t="inlineStr">
@@ -63054,12 +63114,12 @@
       </c>
       <c r="N460" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="O460" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.396</t>
         </is>
       </c>
       <c r="P460" t="inlineStr"/>
@@ -63069,17 +63129,17 @@
       <c r="T460" t="inlineStr"/>
       <c r="U460" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="V460" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="W460" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 24 inch</t>
+          <t>T-Shaped Rubber, 24"</t>
         </is>
       </c>
       <c r="X460" t="inlineStr">
@@ -63094,19 +63154,59 @@
       </c>
       <c r="Z460" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AA460" t="inlineStr"/>
-      <c r="AB460" t="inlineStr"/>
-      <c r="AC460" t="inlineStr"/>
-      <c r="AD460" t="inlineStr"/>
-      <c r="AE460" t="inlineStr"/>
-      <c r="AF460" t="inlineStr"/>
-      <c r="AG460" t="inlineStr"/>
-      <c r="AH460" t="inlineStr"/>
-      <c r="AI460" t="inlineStr"/>
-      <c r="AJ460" t="inlineStr"/>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AA460" t="inlineStr">
+        <is>
+          <t>0.396</t>
+        </is>
+      </c>
+      <c r="AB460" t="inlineStr">
+        <is>
+          <t>Industrial Floor Squeege, Curved, 24"</t>
+        </is>
+      </c>
+      <c r="AC460" t="inlineStr">
+        <is>
+          <t>54524</t>
+        </is>
+      </c>
+      <c r="AD460" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE460" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF460" t="inlineStr">
+        <is>
+          <t>0.390</t>
+        </is>
+      </c>
+      <c r="AG460" t="inlineStr">
+        <is>
+          <t>Industrial Floor Squeege, Straight, 24"</t>
+        </is>
+      </c>
+      <c r="AH460" t="inlineStr">
+        <is>
+          <t>54024</t>
+        </is>
+      </c>
+      <c r="AI460" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ460" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -63628,17 +63728,17 @@
       </c>
       <c r="AF464" t="inlineStr">
         <is>
-          <t>0.412</t>
+          <t>0.407</t>
         </is>
       </c>
       <c r="AG464" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Ettore T-Bar Taper Plastic 18 inch</t>
         </is>
       </c>
       <c r="AH464" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-TAPER-T-BAR-T-BAR-18</t>
         </is>
       </c>
       <c r="AI464" t="inlineStr">
@@ -64624,12 +64724,12 @@
       </c>
       <c r="N471" t="inlineStr">
         <is>
-          <t>0.257</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="O471" t="inlineStr">
         <is>
-          <t>0.239</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="P471" t="inlineStr"/>
@@ -64644,17 +64744,17 @@
       </c>
       <c r="V471" t="inlineStr">
         <is>
-          <t>0.257</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="W471" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 14 inch [Case 36]</t>
         </is>
       </c>
       <c r="X471" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-8</t>
         </is>
       </c>
       <c r="Y471" t="inlineStr">
@@ -64669,17 +64769,17 @@
       </c>
       <c r="AA471" t="inlineStr">
         <is>
-          <t>0.239</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="AB471" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 36 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 06 inch [Case 36]</t>
         </is>
       </c>
       <c r="AC471" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-6</t>
         </is>
       </c>
       <c r="AD471" t="inlineStr">
@@ -64692,31 +64792,11 @@
           <t>1 shared tokens, category fit</t>
         </is>
       </c>
-      <c r="AF471" t="inlineStr">
-        <is>
-          <t>0.239</t>
-        </is>
-      </c>
-      <c r="AG471" t="inlineStr">
-        <is>
-          <t>Sorbo Replacement Rubber Dozen 30 inch</t>
-        </is>
-      </c>
-      <c r="AH471" t="inlineStr">
-        <is>
-          <t>1518</t>
-        </is>
-      </c>
-      <c r="AI471" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AJ471" t="inlineStr">
-        <is>
-          <t>1 shared tokens, category fit</t>
-        </is>
-      </c>
+      <c r="AF471" t="inlineStr"/>
+      <c r="AG471" t="inlineStr"/>
+      <c r="AH471" t="inlineStr"/>
+      <c r="AI471" t="inlineStr"/>
+      <c r="AJ471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -64901,7 +64981,7 @@
       </c>
       <c r="O473" t="inlineStr">
         <is>
-          <t>0.437</t>
+          <t>0.426</t>
         </is>
       </c>
       <c r="P473" t="inlineStr"/>
@@ -64941,17 +65021,17 @@
       </c>
       <c r="AA473" t="inlineStr">
         <is>
-          <t>0.437</t>
+          <t>0.426</t>
         </is>
       </c>
       <c r="AB473" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Ettore T-Bar ProGrip 18 inch</t>
         </is>
       </c>
       <c r="AC473" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-PRO-GRIP-T-BAR-18</t>
         </is>
       </c>
       <c r="AD473" t="inlineStr">
@@ -64961,32 +65041,32 @@
       </c>
       <c r="AE473" t="inlineStr">
         <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF473" t="inlineStr">
+        <is>
+          <t>0.419</t>
+        </is>
+      </c>
+      <c r="AG473" t="inlineStr">
+        <is>
+          <t>Ettore Channel Classic Aluminum 18 inch</t>
+        </is>
+      </c>
+      <c r="AH473" t="inlineStr">
+        <is>
+          <t>1918</t>
+        </is>
+      </c>
+      <c r="AI473" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ473" t="inlineStr">
+        <is>
           <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AF473" t="inlineStr">
-        <is>
-          <t>0.426</t>
-        </is>
-      </c>
-      <c r="AG473" t="inlineStr">
-        <is>
-          <t>Ettore T-Bar ProGrip 18 inch</t>
-        </is>
-      </c>
-      <c r="AH473" t="inlineStr">
-        <is>
-          <t>JRACEN-PRO-GRIP-T-BAR-18</t>
-        </is>
-      </c>
-      <c r="AI473" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AJ473" t="inlineStr">
-        <is>
-          <t>1 shared tokens, category fit</t>
         </is>
       </c>
     </row>
@@ -65054,12 +65134,12 @@
       </c>
       <c r="N474" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="O474" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.396</t>
         </is>
       </c>
       <c r="P474" t="inlineStr"/>
@@ -65069,17 +65149,17 @@
       <c r="T474" t="inlineStr"/>
       <c r="U474" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="V474" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="W474" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 24 inch</t>
+          <t>T-Shaped Rubber, 24"</t>
         </is>
       </c>
       <c r="X474" t="inlineStr">
@@ -65094,19 +65174,59 @@
       </c>
       <c r="Z474" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AA474" t="inlineStr"/>
-      <c r="AB474" t="inlineStr"/>
-      <c r="AC474" t="inlineStr"/>
-      <c r="AD474" t="inlineStr"/>
-      <c r="AE474" t="inlineStr"/>
-      <c r="AF474" t="inlineStr"/>
-      <c r="AG474" t="inlineStr"/>
-      <c r="AH474" t="inlineStr"/>
-      <c r="AI474" t="inlineStr"/>
-      <c r="AJ474" t="inlineStr"/>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AA474" t="inlineStr">
+        <is>
+          <t>0.396</t>
+        </is>
+      </c>
+      <c r="AB474" t="inlineStr">
+        <is>
+          <t>Industrial Floor Squeege, Curved, 24"</t>
+        </is>
+      </c>
+      <c r="AC474" t="inlineStr">
+        <is>
+          <t>54524</t>
+        </is>
+      </c>
+      <c r="AD474" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE474" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF474" t="inlineStr">
+        <is>
+          <t>0.390</t>
+        </is>
+      </c>
+      <c r="AG474" t="inlineStr">
+        <is>
+          <t>Industrial Floor Squeege, Straight, 24"</t>
+        </is>
+      </c>
+      <c r="AH474" t="inlineStr">
+        <is>
+          <t>54024</t>
+        </is>
+      </c>
+      <c r="AI474" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ474" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -65870,12 +65990,12 @@
       </c>
       <c r="N480" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="O480" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.419</t>
         </is>
       </c>
       <c r="P480" t="inlineStr"/>
@@ -65885,17 +66005,17 @@
       <c r="T480" t="inlineStr"/>
       <c r="U480" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
+          <t>1 shared tokens, category fit</t>
         </is>
       </c>
       <c r="V480" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="W480" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>T-Shaped Rubber, 18"</t>
         </is>
       </c>
       <c r="X480" t="inlineStr">
@@ -65910,19 +66030,59 @@
       </c>
       <c r="Z480" t="inlineStr">
         <is>
-          <t>2 shared tokens, category fit</t>
-        </is>
-      </c>
-      <c r="AA480" t="inlineStr"/>
-      <c r="AB480" t="inlineStr"/>
-      <c r="AC480" t="inlineStr"/>
-      <c r="AD480" t="inlineStr"/>
-      <c r="AE480" t="inlineStr"/>
-      <c r="AF480" t="inlineStr"/>
-      <c r="AG480" t="inlineStr"/>
-      <c r="AH480" t="inlineStr"/>
-      <c r="AI480" t="inlineStr"/>
-      <c r="AJ480" t="inlineStr"/>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AA480" t="inlineStr">
+        <is>
+          <t>0.419</t>
+        </is>
+      </c>
+      <c r="AB480" t="inlineStr">
+        <is>
+          <t>Ettore Sleeve Pro+ Microfiber 18 inch</t>
+        </is>
+      </c>
+      <c r="AC480" t="inlineStr">
+        <is>
+          <t>40018</t>
+        </is>
+      </c>
+      <c r="AD480" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AE480" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
+      <c r="AF480" t="inlineStr">
+        <is>
+          <t>0.415</t>
+        </is>
+      </c>
+      <c r="AG480" t="inlineStr">
+        <is>
+          <t>Ettore Squeegee Complete 18</t>
+        </is>
+      </c>
+      <c r="AH480" t="inlineStr">
+        <is>
+          <t>JRACEN-MASTER-BRASS-SQUEEGEES-COMPLET-3</t>
+        </is>
+      </c>
+      <c r="AI480" t="inlineStr">
+        <is>
+          <t>JRacenstein</t>
+        </is>
+      </c>
+      <c r="AJ480" t="inlineStr">
+        <is>
+          <t>1 shared tokens, category fit</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -68265,7 +68425,7 @@
       </c>
       <c r="O497" t="inlineStr">
         <is>
-          <t>0.312</t>
+          <t>0.301</t>
         </is>
       </c>
       <c r="P497" t="inlineStr"/>
@@ -68305,17 +68465,17 @@
       </c>
       <c r="AA497" t="inlineStr">
         <is>
-          <t>0.312</t>
+          <t>0.301</t>
         </is>
       </c>
       <c r="AB497" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Cover for 06in Super Scraper</t>
         </is>
       </c>
       <c r="AC497" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-HEAVY-DUTY-SUPER-SCRAPER-COVER-6</t>
         </is>
       </c>
       <c r="AD497" t="inlineStr">
@@ -68330,17 +68490,17 @@
       </c>
       <c r="AF497" t="inlineStr">
         <is>
-          <t>0.301</t>
+          <t>0.288</t>
         </is>
       </c>
       <c r="AG497" t="inlineStr">
         <is>
-          <t>Cover for 06in Super Scraper</t>
+          <t>Ettore Sleeve Dura 22 inch</t>
         </is>
       </c>
       <c r="AH497" t="inlineStr">
         <is>
-          <t>JRACEN-HEAVY-DUTY-SUPER-SCRAPER-COVER-6</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="AI497" t="inlineStr">
@@ -69542,12 +69702,12 @@
       </c>
       <c r="N506" t="inlineStr">
         <is>
-          <t>0.257</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="O506" t="inlineStr">
         <is>
-          <t>0.239</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="P506" t="inlineStr"/>
@@ -69562,17 +69722,17 @@
       </c>
       <c r="V506" t="inlineStr">
         <is>
-          <t>0.257</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="W506" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Gross 18 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 14 inch [Case 36]</t>
         </is>
       </c>
       <c r="X506" t="inlineStr">
         <is>
-          <t>JRACEN-T-SHAPED-RUBBER-18</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-8</t>
         </is>
       </c>
       <c r="Y506" t="inlineStr">
@@ -69587,17 +69747,17 @@
       </c>
       <c r="AA506" t="inlineStr">
         <is>
-          <t>0.239</t>
+          <t>0.208</t>
         </is>
       </c>
       <c r="AB506" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 36 inch</t>
+          <t>Sorbo Channel Ultralight w/End Clip 06 inch [Case 36]</t>
         </is>
       </c>
       <c r="AC506" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>JRACEN-MASTER-BRASS-CHANNELS-WITH-RUB-6</t>
         </is>
       </c>
       <c r="AD506" t="inlineStr">
@@ -69610,31 +69770,11 @@
           <t>1 shared tokens, category fit</t>
         </is>
       </c>
-      <c r="AF506" t="inlineStr">
-        <is>
-          <t>0.239</t>
-        </is>
-      </c>
-      <c r="AG506" t="inlineStr">
-        <is>
-          <t>Sorbo Replacement Rubber Dozen 30 inch</t>
-        </is>
-      </c>
-      <c r="AH506" t="inlineStr">
-        <is>
-          <t>1518</t>
-        </is>
-      </c>
-      <c r="AI506" t="inlineStr">
-        <is>
-          <t>JRacenstein</t>
-        </is>
-      </c>
-      <c r="AJ506" t="inlineStr">
-        <is>
-          <t>1 shared tokens, category fit</t>
-        </is>
-      </c>
+      <c r="AF506" t="inlineStr"/>
+      <c r="AG506" t="inlineStr"/>
+      <c r="AH506" t="inlineStr"/>
+      <c r="AI506" t="inlineStr"/>
+      <c r="AJ506" t="inlineStr"/>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
@@ -72268,7 +72408,7 @@
       </c>
       <c r="N527" t="inlineStr">
         <is>
-          <t>0.471</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="O527" t="inlineStr">
@@ -72288,12 +72428,12 @@
       </c>
       <c r="V527" t="inlineStr">
         <is>
-          <t>0.471</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="W527" t="inlineStr">
         <is>
-          <t>Sorbo Replacement Rubber Dozen 14 inch</t>
+          <t>T-Shaped Rubber, 14"</t>
         </is>
       </c>
       <c r="X527" t="inlineStr">

</xml_diff>